<commit_message>
feat: boton limpiar seleccionado en modales de importar farmacias y turnos
</commit_message>
<xml_diff>
--- a/public/plantilla-turnos.xlsx
+++ b/public/plantilla-turnos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Harold Besson\Desktop\CODE\farmaguardia\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Harold Besson\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BBB4D6D-6A8F-4AA7-9287-D19EF325F94B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D4A17CF-74AE-4993-A31B-9321E5487446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>farmacia</t>
   </si>
@@ -43,6 +43,12 @@
   </si>
   <si>
     <t>Farma Descuento Ayacucho Plus</t>
+  </si>
+  <si>
+    <t>08:00</t>
+  </si>
+  <si>
+    <t>2026-08-02</t>
   </si>
 </sst>
 </file>
@@ -78,10 +84,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -366,6 +371,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
   </cols>
   <sheetData>
@@ -387,17 +393,17 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C2" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.33333333333333331</v>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>